<commit_message>
Update Scenario 1 files with public permissions
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Contoso_Outage_Restoration_Tracker.xlsx
+++ b/Contoso_Outage_Restoration_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_28434487EC5E77E93A92FB8A0C48C139C92C4702" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_28434487EC5E77E93A92FB8A0C48C139C92C4702" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E625637B-4FF7-4FDE-97C1-A123210EB49D}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,10 +11,21 @@
     <sheet name="Outage Log" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1710,21 +1721,21 @@
       <c r="C31" s="29"/>
       <c r="D31" s="29"/>
       <c r="E31" s="29"/>
-      <c r="F31" s="10" t="str">
+      <c r="F31" s="10">
         <f>SUM(F5:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="11" t="str">
+        <v>249490</v>
+      </c>
+      <c r="G31" s="11">
         <f>SUM(G5:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="12" t="str">
+        <v>197</v>
+      </c>
+      <c r="H31" s="12">
         <f>AVERAGE(H5:H30)</f>
-        <v/>
-      </c>
-      <c r="I31" s="12" t="str">
+        <v>8.615384615384615</v>
+      </c>
+      <c r="I31" s="12">
         <f>AVERAGEIF(I5:I30,"&gt;0")</f>
-        <v/>
+        <v>9.5749999999999993</v>
       </c>
       <c r="J31" s="13"/>
     </row>
@@ -1781,9 +1792,9 @@
       </c>
       <c r="B5" s="30"/>
       <c r="C5" s="30"/>
-      <c r="D5" s="17" t="str">
+      <c r="D5" s="17">
         <f>COUNTA('Outage Log'!A5:A30)</f>
-        <v/>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1792,9 +1803,9 @@
       </c>
       <c r="B6" s="30"/>
       <c r="C6" s="30"/>
-      <c r="D6" s="17" t="str">
+      <c r="D6" s="17">
         <f>SUM('Outage Log'!F5:F30)</f>
-        <v/>
+        <v>249490</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1803,9 +1814,9 @@
       </c>
       <c r="B7" s="30"/>
       <c r="C7" s="30"/>
-      <c r="D7" s="17" t="str">
+      <c r="D7" s="17">
         <f>MAX('Outage Log'!F5:F30)</f>
-        <v/>
+        <v>41200</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1814,9 +1825,9 @@
       </c>
       <c r="B8" s="30"/>
       <c r="C8" s="30"/>
-      <c r="D8" s="17" t="str">
+      <c r="D8" s="17">
         <f>SUM('Outage Log'!G5:G30)</f>
-        <v/>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1825,9 +1836,9 @@
       </c>
       <c r="B9" s="30"/>
       <c r="C9" s="30"/>
-      <c r="D9" s="18" t="str">
+      <c r="D9" s="18">
         <f>AVERAGEIF('Outage Log'!I5:I30,"&gt;0")</f>
-        <v/>
+        <v>9.5749999999999993</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1836,9 +1847,9 @@
       </c>
       <c r="B10" s="30"/>
       <c r="C10" s="30"/>
-      <c r="D10" s="17" t="str">
+      <c r="D10" s="17">
         <f>COUNTIF('Outage Log'!J5:J30,"In Progress")</f>
-        <v/>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1864,98 +1875,98 @@
       <c r="A14" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="19" t="str">
+      <c r="B14" s="19">
         <f>COUNTIF('Outage Log'!C5:C30,A14)</f>
-        <v/>
-      </c>
-      <c r="C14" s="20" t="str">
+        <v>4</v>
+      </c>
+      <c r="C14" s="20">
         <f>SUMIF('Outage Log'!C5:C30,A14,'Outage Log'!F5:F30)</f>
-        <v/>
-      </c>
-      <c r="D14" s="21" t="str">
+        <v>11280</v>
+      </c>
+      <c r="D14" s="21">
         <f>IFERROR(AVERAGEIFS('Outage Log'!I5:I30,'Outage Log'!C5:C30,A14,'Outage Log'!I5:I30,"&gt;0"),"-")</f>
-        <v/>
+        <v>4.166666666666667</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="19" t="str">
+      <c r="B15" s="19">
         <f>COUNTIF('Outage Log'!C5:C30,A15)</f>
-        <v/>
-      </c>
-      <c r="C15" s="20" t="str">
+        <v>8</v>
+      </c>
+      <c r="C15" s="20">
         <f>SUMIF('Outage Log'!C5:C30,A15,'Outage Log'!F5:F30)</f>
-        <v/>
-      </c>
-      <c r="D15" s="21" t="str">
+        <v>138430</v>
+      </c>
+      <c r="D15" s="21">
         <f>IFERROR(AVERAGEIFS('Outage Log'!I5:I30,'Outage Log'!C5:C30,A15,'Outage Log'!I5:I30,"&gt;0"),"-")</f>
-        <v/>
+        <v>13.285714285714286</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="19" t="str">
+      <c r="B16" s="19">
         <f>COUNTIF('Outage Log'!C5:C30,A16)</f>
-        <v/>
-      </c>
-      <c r="C16" s="20" t="str">
+        <v>5</v>
+      </c>
+      <c r="C16" s="20">
         <f>SUMIF('Outage Log'!C5:C30,A16,'Outage Log'!F5:F30)</f>
-        <v/>
-      </c>
-      <c r="D16" s="21" t="str">
+        <v>32370</v>
+      </c>
+      <c r="D16" s="21">
         <f>IFERROR(AVERAGEIFS('Outage Log'!I5:I30,'Outage Log'!C5:C30,A16,'Outage Log'!I5:I30,"&gt;0"),"-")</f>
-        <v/>
+        <v>8.5</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="19" t="str">
+      <c r="B17" s="19">
         <f>COUNTIF('Outage Log'!C5:C30,A17)</f>
-        <v/>
-      </c>
-      <c r="C17" s="20" t="str">
+        <v>3</v>
+      </c>
+      <c r="C17" s="20">
         <f>SUMIF('Outage Log'!C5:C30,A17,'Outage Log'!F5:F30)</f>
-        <v/>
-      </c>
-      <c r="D17" s="21" t="str">
+        <v>15710</v>
+      </c>
+      <c r="D17" s="21">
         <f>IFERROR(AVERAGEIFS('Outage Log'!I5:I30,'Outage Log'!C5:C30,A17,'Outage Log'!I5:I30,"&gt;0"),"-")</f>
-        <v/>
+        <v>5.25</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="19" t="str">
+      <c r="B18" s="19">
         <f>COUNTIF('Outage Log'!C5:C30,A18)</f>
-        <v/>
-      </c>
-      <c r="C18" s="20" t="str">
+        <v>6</v>
+      </c>
+      <c r="C18" s="20">
         <f>SUMIF('Outage Log'!C5:C30,A18,'Outage Log'!F5:F30)</f>
-        <v/>
-      </c>
-      <c r="D18" s="21" t="str">
+        <v>51700</v>
+      </c>
+      <c r="D18" s="21">
         <f>IFERROR(AVERAGEIFS('Outage Log'!I5:I30,'Outage Log'!C5:C30,A18,'Outage Log'!I5:I30,"&gt;0"),"-")</f>
-        <v/>
+        <v>10.375</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="11" t="str">
+      <c r="B19" s="11">
         <f>SUM(B14:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="23" t="str">
+        <v>26</v>
+      </c>
+      <c r="C19" s="23">
         <f>SUM(C14:C18)</f>
-        <v/>
+        <v>249490</v>
       </c>
       <c r="D19" s="11"/>
     </row>
@@ -1979,65 +1990,65 @@
       <c r="A23" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="19" t="str">
+      <c r="B23" s="19">
         <f>COUNTIF('Outage Log'!E5:E30,A23)</f>
-        <v/>
-      </c>
-      <c r="C23" s="20" t="str">
+        <v>9</v>
+      </c>
+      <c r="C23" s="20">
         <f>SUMIF('Outage Log'!E5:E30,A23,'Outage Log'!F5:F30)</f>
-        <v/>
+        <v>104720</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="19" t="str">
+      <c r="B24" s="19">
         <f>COUNTIF('Outage Log'!E5:E30,A24)</f>
-        <v/>
-      </c>
-      <c r="C24" s="20" t="str">
+        <v>4</v>
+      </c>
+      <c r="C24" s="20">
         <f>SUMIF('Outage Log'!E5:E30,A24,'Outage Log'!F5:F30)</f>
-        <v/>
+        <v>105230</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="19" t="str">
+      <c r="B25" s="19">
         <f>COUNTIF('Outage Log'!E5:E30,A25)</f>
-        <v/>
-      </c>
-      <c r="C25" s="20" t="str">
+        <v>5</v>
+      </c>
+      <c r="C25" s="20">
         <f>SUMIF('Outage Log'!E5:E30,A25,'Outage Log'!F5:F30)</f>
-        <v/>
+        <v>24160</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="19" t="str">
+      <c r="B26" s="19">
         <f>COUNTIF('Outage Log'!E5:E30,A26)</f>
-        <v/>
-      </c>
-      <c r="C26" s="20" t="str">
+        <v>6</v>
+      </c>
+      <c r="C26" s="20">
         <f>SUMIF('Outage Log'!E5:E30,A26,'Outage Log'!F5:F30)</f>
-        <v/>
+        <v>14080</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="19" t="str">
+      <c r="B27" s="19">
         <f>COUNTIF('Outage Log'!E5:E30,A27)</f>
-        <v/>
-      </c>
-      <c r="C27" s="20" t="str">
+        <v>2</v>
+      </c>
+      <c r="C27" s="20">
         <f>SUMIF('Outage Log'!E5:E30,A27,'Outage Log'!F5:F30)</f>
-        <v/>
+        <v>1300</v>
       </c>
     </row>
   </sheetData>
@@ -2057,6 +2068,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" removed="0"/>
+  <clbl:label id="{87867195-f2b8-4ac2-b0b6-6bb73cb33afc}" enabled="1" method="Privileged" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>